<commit_message>
Mastersheet: röd markering av tak-bindande kapaciteter + batch17-rapport
build_mastersheet.py: _binds()/binds_dict() flaggar kraftslag där p_nom_opt ≈
p_nom_max (bara extendable; zon + Norden-aggregat) → röd font i Kapacitet-blocket
(49 celler i batch 17, bekräftar t.ex. SE-S sol 24 GW + SE-N onshore 20.4 GW vid tak).
docs/batch17_rapport.md: bloggformat-rapport om baseline + 5 varianter (run170-175).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/batch17_mastersheet.xlsx
+++ b/docs/batch17_mastersheet.xlsx
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <color rgb="FFCC0000"/>
     </font>
   </fonts>
   <fills count="2">
@@ -47,8 +50,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -650,7 +654,7 @@
       <c r="E4" t="n">
         <v>0</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="1" t="n">
         <v>20.39</v>
       </c>
       <c r="G4" t="n">
@@ -756,13 +760,13 @@
       <c r="E5" t="n">
         <v>6.9</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="1" t="n">
         <v>14.38</v>
       </c>
       <c r="G5" t="n">
         <v>0.13</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="1" t="n">
         <v>24</v>
       </c>
       <c r="I5" t="n">
@@ -862,13 +866,13 @@
       <c r="E6" t="n">
         <v>0</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="1" t="n">
         <v>5.54</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="1" t="n">
         <v>1.67</v>
       </c>
       <c r="I6" t="n">
@@ -968,7 +972,7 @@
       <c r="E7" t="n">
         <v>0</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="1" t="n">
         <v>3.73</v>
       </c>
       <c r="G7" t="n">
@@ -1074,7 +1078,7 @@
       <c r="E8" t="n">
         <v>0</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="1" t="n">
         <v>6.76</v>
       </c>
       <c r="G8" t="n">
@@ -1395,7 +1399,7 @@
       <c r="E11" t="n">
         <v>0</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" s="1" t="n">
         <v>20.39</v>
       </c>
       <c r="G11" t="n">
@@ -1501,7 +1505,7 @@
       <c r="E12" t="n">
         <v>8.4</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12" s="1" t="n">
         <v>14.38</v>
       </c>
       <c r="G12" t="n">
@@ -1607,13 +1611,13 @@
       <c r="E13" t="n">
         <v>0</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13" s="1" t="n">
         <v>5.54</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
       </c>
-      <c r="H13" t="n">
+      <c r="H13" s="1" t="n">
         <v>1.67</v>
       </c>
       <c r="I13" t="n">
@@ -1713,7 +1717,7 @@
       <c r="E14" t="n">
         <v>0</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14" s="1" t="n">
         <v>3.73</v>
       </c>
       <c r="G14" t="n">
@@ -1819,7 +1823,7 @@
       <c r="E15" t="n">
         <v>0</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15" s="1" t="n">
         <v>6.76</v>
       </c>
       <c r="G15" t="n">
@@ -2140,7 +2144,7 @@
       <c r="E18" t="n">
         <v>0</v>
       </c>
-      <c r="F18" t="n">
+      <c r="F18" s="1" t="n">
         <v>20.39</v>
       </c>
       <c r="G18" t="n">
@@ -2246,7 +2250,7 @@
       <c r="E19" t="n">
         <v>11.13</v>
       </c>
-      <c r="F19" t="n">
+      <c r="F19" s="1" t="n">
         <v>14.38</v>
       </c>
       <c r="G19" t="n">
@@ -2352,7 +2356,7 @@
       <c r="E20" t="n">
         <v>0</v>
       </c>
-      <c r="F20" t="n">
+      <c r="F20" s="1" t="n">
         <v>5.54</v>
       </c>
       <c r="G20" t="n">
@@ -2458,7 +2462,7 @@
       <c r="E21" t="n">
         <v>0</v>
       </c>
-      <c r="F21" t="n">
+      <c r="F21" s="1" t="n">
         <v>3.73</v>
       </c>
       <c r="G21" t="n">
@@ -2564,7 +2568,7 @@
       <c r="E22" t="n">
         <v>0</v>
       </c>
-      <c r="F22" t="n">
+      <c r="F22" s="1" t="n">
         <v>6.76</v>
       </c>
       <c r="G22" t="n">
@@ -2885,13 +2889,13 @@
       <c r="E25" t="n">
         <v>0</v>
       </c>
-      <c r="F25" t="n">
+      <c r="F25" s="1" t="n">
         <v>16.32</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
       </c>
-      <c r="H25" t="n">
+      <c r="H25" s="1" t="n">
         <v>1.28</v>
       </c>
       <c r="I25" t="n">
@@ -2991,13 +2995,13 @@
       <c r="E26" t="n">
         <v>6.9</v>
       </c>
-      <c r="F26" t="n">
+      <c r="F26" s="1" t="n">
         <v>11.5</v>
       </c>
       <c r="G26" t="n">
         <v>2.9</v>
       </c>
-      <c r="H26" t="n">
+      <c r="H26" s="1" t="n">
         <v>24</v>
       </c>
       <c r="I26" t="n">
@@ -3097,13 +3101,13 @@
       <c r="E27" t="n">
         <v>0</v>
       </c>
-      <c r="F27" t="n">
+      <c r="F27" s="1" t="n">
         <v>4.43</v>
       </c>
       <c r="G27" t="n">
         <v>0</v>
       </c>
-      <c r="H27" t="n">
+      <c r="H27" s="1" t="n">
         <v>1.67</v>
       </c>
       <c r="I27" t="n">
@@ -3203,7 +3207,7 @@
       <c r="E28" t="n">
         <v>0</v>
       </c>
-      <c r="F28" t="n">
+      <c r="F28" s="1" t="n">
         <v>2.98</v>
       </c>
       <c r="G28" t="n">
@@ -3309,13 +3313,13 @@
       <c r="E29" t="n">
         <v>0</v>
       </c>
-      <c r="F29" t="n">
+      <c r="F29" s="1" t="n">
         <v>5.46</v>
       </c>
       <c r="G29" t="n">
         <v>2.61</v>
       </c>
-      <c r="H29" t="n">
+      <c r="H29" s="1" t="n">
         <v>32.83</v>
       </c>
       <c r="I29" t="n">
@@ -3415,7 +3419,7 @@
       <c r="E30" t="n">
         <v>5.52</v>
       </c>
-      <c r="F30" t="n">
+      <c r="F30" s="1" t="n">
         <v>22.58</v>
       </c>
       <c r="G30" t="n">
@@ -3519,7 +3523,7 @@
       <c r="E31" t="n">
         <v>12.42</v>
       </c>
-      <c r="F31" t="n">
+      <c r="F31" s="1" t="n">
         <v>63.26</v>
       </c>
       <c r="G31" t="n">
@@ -3630,13 +3634,13 @@
       <c r="E32" t="n">
         <v>0</v>
       </c>
-      <c r="F32" t="n">
+      <c r="F32" s="1" t="n">
         <v>20.39</v>
       </c>
       <c r="G32" t="n">
         <v>0</v>
       </c>
-      <c r="H32" t="n">
+      <c r="H32" s="1" t="n">
         <v>1.28</v>
       </c>
       <c r="I32" t="n">
@@ -3736,13 +3740,13 @@
       <c r="E33" t="n">
         <v>6.9</v>
       </c>
-      <c r="F33" t="n">
+      <c r="F33" s="1" t="n">
         <v>14.38</v>
       </c>
       <c r="G33" t="n">
         <v>0.53</v>
       </c>
-      <c r="H33" t="n">
+      <c r="H33" s="1" t="n">
         <v>24</v>
       </c>
       <c r="I33" t="n">
@@ -3842,13 +3846,13 @@
       <c r="E34" t="n">
         <v>0</v>
       </c>
-      <c r="F34" t="n">
+      <c r="F34" s="1" t="n">
         <v>5.54</v>
       </c>
       <c r="G34" t="n">
         <v>0</v>
       </c>
-      <c r="H34" t="n">
+      <c r="H34" s="1" t="n">
         <v>1.67</v>
       </c>
       <c r="I34" t="n">
@@ -3948,10 +3952,10 @@
       <c r="E35" t="n">
         <v>0</v>
       </c>
-      <c r="F35" t="n">
+      <c r="F35" s="1" t="n">
         <v>3.73</v>
       </c>
-      <c r="G35" t="n">
+      <c r="G35" s="1" t="n">
         <v>4.87</v>
       </c>
       <c r="H35" t="n">
@@ -4054,7 +4058,7 @@
       <c r="E36" t="n">
         <v>0</v>
       </c>
-      <c r="F36" t="n">
+      <c r="F36" s="1" t="n">
         <v>6.76</v>
       </c>
       <c r="G36" t="n">
@@ -4160,7 +4164,7 @@
       <c r="E37" t="n">
         <v>4.4</v>
       </c>
-      <c r="F37" t="n">
+      <c r="F37" s="1" t="n">
         <v>28.22</v>
       </c>
       <c r="G37" t="n">
@@ -4264,7 +4268,7 @@
       <c r="E38" t="n">
         <v>11.3</v>
       </c>
-      <c r="F38" t="n">
+      <c r="F38" s="1" t="n">
         <v>79.01000000000001</v>
       </c>
       <c r="G38" t="n">
@@ -4375,13 +4379,13 @@
       <c r="E39" t="n">
         <v>0</v>
       </c>
-      <c r="F39" t="n">
+      <c r="F39" s="1" t="n">
         <v>20.39</v>
       </c>
       <c r="G39" t="n">
         <v>0</v>
       </c>
-      <c r="H39" t="n">
+      <c r="H39" s="1" t="n">
         <v>1.28</v>
       </c>
       <c r="I39" t="n">
@@ -4481,13 +4485,13 @@
       <c r="E40" t="n">
         <v>6.9</v>
       </c>
-      <c r="F40" t="n">
+      <c r="F40" s="1" t="n">
         <v>14.38</v>
       </c>
       <c r="G40" t="n">
         <v>0.13</v>
       </c>
-      <c r="H40" t="n">
+      <c r="H40" s="1" t="n">
         <v>24</v>
       </c>
       <c r="I40" t="n">
@@ -4587,13 +4591,13 @@
       <c r="E41" t="n">
         <v>0</v>
       </c>
-      <c r="F41" t="n">
+      <c r="F41" s="1" t="n">
         <v>5.54</v>
       </c>
       <c r="G41" t="n">
         <v>0</v>
       </c>
-      <c r="H41" t="n">
+      <c r="H41" s="1" t="n">
         <v>1.67</v>
       </c>
       <c r="I41" t="n">
@@ -4693,7 +4697,7 @@
       <c r="E42" t="n">
         <v>0</v>
       </c>
-      <c r="F42" t="n">
+      <c r="F42" s="1" t="n">
         <v>3.73</v>
       </c>
       <c r="G42" t="n">
@@ -4799,13 +4803,13 @@
       <c r="E43" t="n">
         <v>0</v>
       </c>
-      <c r="F43" t="n">
+      <c r="F43" s="1" t="n">
         <v>6.76</v>
       </c>
       <c r="G43" t="n">
         <v>2.61</v>
       </c>
-      <c r="H43" t="n">
+      <c r="H43" s="1" t="n">
         <v>32.84</v>
       </c>
       <c r="I43" t="n">

</xml_diff>